<commit_message>
Add Site Lens record.
</commit_message>
<xml_diff>
--- a/Site Lens/DS/SiteLens.xlsx
+++ b/Site Lens/DS/SiteLens.xlsx
@@ -70,7 +70,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">demo-001</t>
+          <t xml:space="preserve">6da63e65-4794-44e2-8b5c-25e07d2b217a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -80,27 +80,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">电缆桥架固定件松动</t>
+          <t xml:space="preserve">test</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">二层东侧走廊发现一处桥架固定件松动，轻微晃动。建议检查相邻固定点并重新紧固。</t>
+          <t xml:space="preserve">test</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Building A · Level 2</t>
+          <t xml:space="preserve">地点待补充</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">高</t>
+          <t xml:space="preserve">中</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">处理中</t>
+          <t xml:space="preserve">新建</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -110,7 +110,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17T09:10:00.000Z</t>
+          <t xml:space="preserve">2026-10-17T12:59:43.540Z</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -127,7 +127,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">demo-002</t>
+          <t xml:space="preserve">demo-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -137,27 +137,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备间安全标识缺失</t>
+          <t xml:space="preserve">电缆桥架固定件松动</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备间入口处未发现安全警示标识。</t>
+          <t xml:space="preserve">二层东侧走廊发现一处桥架固定件松动，轻微晃动。建议检查相邻固定点并重新紧固。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Building A · Equipment Room</t>
+          <t xml:space="preserve">Building A · Level 2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">高</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">新建</t>
+          <t xml:space="preserve">处理中</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -167,7 +167,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17T08:42:00.000Z</t>
+          <t xml:space="preserve">2026-10-17T09:10:00.000Z</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -184,55 +184,112 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t xml:space="preserve">demo-002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SGP Project</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设备间安全标识缺失</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设备间入口处未发现安全警示标识。</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Building A · Equipment Room</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新建</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Michael Shi</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-17T08:42:00.000Z</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t xml:space="preserve">demo-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t xml:space="preserve">SGP Project</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t xml:space="preserve">地面排水口需要清理</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">走廊排水口有少量施工碎屑，建议清理后复查排水情况。</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t xml:space="preserve">West Wing · Ground Floor</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t xml:space="preserve">低</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t xml:space="preserve">已解决</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t xml:space="preserve">Michael Shi</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-15T14:20:00.000Z</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Delete Site Lens record.
</commit_message>
<xml_diff>
--- a/Site Lens/DS/SiteLens.xlsx
+++ b/Site Lens/DS/SiteLens.xlsx
@@ -70,7 +70,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30a0b177-1417-45e2-9b03-5d36cb627ad3</t>
+          <t xml:space="preserve">6da63e65-4794-44e2-8b5c-25e07d2b217a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -80,12 +80,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">test 2</t>
+          <t xml:space="preserve">test</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">test 2</t>
+          <t xml:space="preserve">test</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -110,7 +110,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17T13:00:13.631Z</t>
+          <t xml:space="preserve">2026-10-17T12:59:43.540Z</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -127,7 +127,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6da63e65-4794-44e2-8b5c-25e07d2b217a</t>
+          <t xml:space="preserve">demo-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -137,27 +137,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">test</t>
+          <t xml:space="preserve">电缆桥架固定件松动</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">test</t>
+          <t xml:space="preserve">二层东侧走廊发现一处桥架固定件松动，轻微晃动。建议检查相邻固定点并重新紧固。</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">地点待补充</t>
+          <t xml:space="preserve">Building A · Level 2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">高</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">新建</t>
+          <t xml:space="preserve">处理中</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -167,7 +167,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17T12:59:43.540Z</t>
+          <t xml:space="preserve">2026-10-17T09:10:00.000Z</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -184,7 +184,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">demo-001</t>
+          <t xml:space="preserve">demo-002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -194,27 +194,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">电缆桥架固定件松动</t>
+          <t xml:space="preserve">设备间安全标识缺失</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">二层东侧走廊发现一处桥架固定件松动，轻微晃动。建议检查相邻固定点并重新紧固。</t>
+          <t xml:space="preserve">设备间入口处未发现安全警示标识。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Building A · Level 2</t>
+          <t xml:space="preserve">Building A · Equipment Room</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">高</t>
+          <t xml:space="preserve">中</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">处理中</t>
+          <t xml:space="preserve">新建</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -224,7 +224,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17T09:10:00.000Z</t>
+          <t xml:space="preserve">2026-10-17T08:42:00.000Z</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -241,7 +241,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">demo-002</t>
+          <t xml:space="preserve">demo-003</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -251,27 +251,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备间安全标识缺失</t>
+          <t xml:space="preserve">地面排水口需要清理</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备间入口处未发现安全警示标识。</t>
+          <t xml:space="preserve">走廊排水口有少量施工碎屑，建议清理后复查排水情况。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Building A · Equipment Room</t>
+          <t xml:space="preserve">West Wing · Ground Floor</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">中</t>
+          <t xml:space="preserve">低</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">新建</t>
+          <t xml:space="preserve">已解决</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -281,7 +281,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-17T08:42:00.000Z</t>
+          <t xml:space="preserve">2026-10-15T14:20:00.000Z</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -290,63 +290,6 @@
         </is>
       </c>
       <c r="K5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">demo-003</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SGP Project</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地面排水口需要清理</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">走廊排水口有少量施工碎屑，建议清理后复查排水情况。</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">West Wing · Ground Floor</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">低</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已解决</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Michael Shi</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-15T14:20:00.000Z</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Update Site Lens record.
</commit_message>
<xml_diff>
--- a/Site Lens/DS/SiteLens.xlsx
+++ b/Site Lens/DS/SiteLens.xlsx
@@ -127,64 +127,64 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">记录ID</t>
+          <t xml:space="preserve">BCF9F1A3-25D1-4C14-BA8C-DA1EAD4D54CA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">项目</t>
+          <t xml:space="preserve">SGP Project</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">标题</t>
+          <t xml:space="preserve">测试</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">描述 / 语音转写</t>
+          <t xml:space="preserve">开始测试</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">地点</t>
+          <t xml:space="preserve">地点待补充</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">优先级</t>
+          <t xml:space="preserve">中</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">状态</t>
+          <t xml:space="preserve">新建</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">记录人</t>
+          <t xml:space="preserve">Michael Shi</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">记录时间</t>
+          <t xml:space="preserve">2026-10-19T13:30:42Z</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">照片路径</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">语音路径</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BCF9F1A3-25D1-4C14-BA8C-DA1EAD4D54CA</t>
+          <t xml:space="preserve">demo-002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -194,17 +194,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">测试</t>
+          <t xml:space="preserve">设备间安全标识缺失</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">开始测试</t>
+          <t xml:space="preserve">设备间入口处未发现安全警示标识。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">地点待补充</t>
+          <t xml:space="preserve">Building A · Equipment Room</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -224,7 +224,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19T13:30:42Z</t>
+          <t xml:space="preserve">2026-10-17T08:42:00.000Z</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -233,63 +233,6 @@
         </is>
       </c>
       <c r="K4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">demo-002</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SGP Project</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设备间安全标识缺失</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设备间入口处未发现安全警示标识。</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Building A · Equipment Room</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">新建</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Michael Shi</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-17T08:42:00.000Z</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>